<commit_message>
week 01: complete day 04 Excel, Python, and JOIN exercises
</commit_message>
<xml_diff>
--- a/practice/week01/day03/excel_practice.xlsx
+++ b/practice/week01/day03/excel_practice.xlsx
@@ -2,22 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Codex\study\practice\week01\day03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A432636C-C6E9-4FF7-A0BA-96483B7B453F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6F2E1CF-4D6D-4A7D-BD0A-EE35AEC47131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="订单数据" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId1"/>
+    <sheet name="订单数据" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId2"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="18">
   <si>
     <t>customer</t>
   </si>
@@ -96,7 +97,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -106,6 +107,11 @@
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -140,7 +146,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -161,7 +167,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="跳跳虎武大郎打" refreshedDate="46309.934118865742" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="6" xr:uid="{3C88854E-3BFB-4E69-869E-75938914C496}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="跳跳虎武大郎打" refreshedDate="46310.875209375001" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="6" xr:uid="{454124B6-DD78-4DF5-96C3-B1CF008052F9}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:D7" sheet="订单数据"/>
   </cacheSource>
@@ -180,7 +186,10 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="80" maxValue="300"/>
     </cacheField>
     <cacheField name="status" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="2">
+        <s v="paid"/>
+        <s v="refunded"/>
+      </sharedItems>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -197,44 +206,44 @@
     <s v="张三"/>
     <x v="0"/>
     <n v="120"/>
-    <s v="paid"/>
+    <x v="0"/>
   </r>
   <r>
     <s v="李四"/>
     <x v="1"/>
     <n v="80"/>
-    <s v="paid"/>
+    <x v="0"/>
   </r>
   <r>
     <s v="王五"/>
     <x v="0"/>
     <n v="200"/>
-    <s v="refunded"/>
+    <x v="1"/>
   </r>
   <r>
     <s v="赵六"/>
     <x v="0"/>
     <n v="150"/>
-    <s v="paid"/>
+    <x v="0"/>
   </r>
   <r>
     <s v="孙七"/>
     <x v="2"/>
     <n v="90"/>
-    <s v="paid"/>
+    <x v="0"/>
   </r>
   <r>
     <s v="周八"/>
     <x v="1"/>
     <n v="300"/>
-    <s v="paid"/>
+    <x v="0"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8FE1CCDB-B153-4740-A051-C36E9426ABC5}" name="数据透视表1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A10:B14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{431D4976-7845-4D85-B70C-4C458D8858F3}" name="数据透视表7" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="值" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="4">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
@@ -246,7 +255,13 @@
       </items>
     </pivotField>
     <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
   </pivotFields>
   <rowFields count="1">
     <field x="1"/>
@@ -268,6 +283,9 @@
   <colItems count="1">
     <i/>
   </colItems>
+  <pageFields count="1">
+    <pageField fld="3" item="0" hier="-1"/>
+  </pageFields>
   <dataFields count="1">
     <dataField name="求和项:amount" fld="2" baseField="0" baseItem="0"/>
   </dataFields>
@@ -599,17 +617,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62136EB9-E748-4DFF-AE7A-9DB63D5D0CCF}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7">
+        <v>740</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -623,7 +706,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="11.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -636,8 +719,15 @@
       <c r="D2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="str">
+        <f>_xlfn.XLOOKUP(F2,A:A,B:B)</f>
+        <v>上海</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -650,8 +740,15 @@
       <c r="D3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="F3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" t="str">
+        <f>_xlfn.XLOOKUP(F3,A:A,B:B)</f>
+        <v>北京</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -664,8 +761,15 @@
       <c r="D4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="str">
+        <f>_xlfn.XLOOKUP(F4,A:A,B:B)</f>
+        <v>上海</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -678,8 +782,15 @@
       <c r="D5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="str">
+        <f>_xlfn.XLOOKUP(F5,A:A,B:B)</f>
+        <v>上海</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -692,8 +803,15 @@
       <c r="D6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="str">
+        <f>_xlfn.XLOOKUP(F6,A:A,B:B)</f>
+        <v>深圳</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -706,103 +824,18 @@
       <c r="D7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10">
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="str">
+        <f>_xlfn.XLOOKUP(F7,A:A,B:B)</f>
+        <v>北京</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="D10" s="3">
         <f>SUMIF($D$2:$D$7,"paid",$C$2:$C$7)</f>
         <v>740</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="3">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="3">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="3">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="3">
-        <v>940</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B16" t="str">
-        <f>VLOOKUP(A2,$A$2:$D$7,2,FALSE)</f>
-        <v>上海</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" t="str">
-        <f t="shared" ref="B17:B21" si="0">VLOOKUP(A3,$A$2:$D$7,2,FALSE)</f>
-        <v>北京</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" t="str">
-        <f t="shared" si="0"/>
-        <v>上海</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" t="str">
-        <f t="shared" si="0"/>
-        <v>上海</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" t="str">
-        <f t="shared" si="0"/>
-        <v>深圳</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" t="str">
-        <f t="shared" si="0"/>
-        <v>北京</v>
       </c>
     </row>
   </sheetData>

</xml_diff>